<commit_message>
reanalyzed full dataset QC metrics
</commit_message>
<xml_diff>
--- a/fullDataset/proportions/FLCvNML_cells_per_cluster.xlsx
+++ b/fullDataset/proportions/FLCvNML_cells_per_cluster.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -55,12 +55,6 @@
   </si>
   <si>
     <t xml:space="preserve">10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12</t>
   </si>
 </sst>
 </file>
@@ -405,10 +399,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>24019</v>
+        <v>22982</v>
       </c>
       <c r="C2" t="n">
-        <v>10990</v>
+        <v>12208</v>
       </c>
     </row>
     <row r="3">
@@ -416,10 +410,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>11314</v>
+        <v>11740</v>
       </c>
       <c r="C3" t="n">
-        <v>4881</v>
+        <v>3138</v>
       </c>
     </row>
     <row r="4">
@@ -427,10 +421,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>8318</v>
+        <v>8889</v>
       </c>
       <c r="C4" t="n">
-        <v>5633</v>
+        <v>5581</v>
       </c>
     </row>
     <row r="5">
@@ -438,10 +432,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>9426</v>
+        <v>9404</v>
       </c>
       <c r="C5" t="n">
-        <v>3354</v>
+        <v>2006</v>
       </c>
     </row>
     <row r="6">
@@ -449,10 +443,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>7425</v>
+        <v>8511</v>
       </c>
       <c r="C6" t="n">
-        <v>4009</v>
+        <v>1747</v>
       </c>
     </row>
     <row r="7">
@@ -460,10 +454,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>8067</v>
+        <v>7772</v>
       </c>
       <c r="C7" t="n">
-        <v>2185</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8">
@@ -471,10 +465,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>4501</v>
+        <v>5091</v>
       </c>
       <c r="C8" t="n">
-        <v>3484</v>
+        <v>2317</v>
       </c>
     </row>
     <row r="9">
@@ -482,10 +476,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>1727</v>
+        <v>1849</v>
       </c>
       <c r="C9" t="n">
-        <v>5232</v>
+        <v>4080</v>
       </c>
     </row>
     <row r="10">
@@ -493,10 +487,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>3631</v>
+        <v>3517</v>
       </c>
       <c r="C10" t="n">
-        <v>3282</v>
+        <v>1530</v>
       </c>
     </row>
     <row r="11">
@@ -504,10 +498,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>79</v>
+        <v>2150</v>
       </c>
       <c r="C11" t="n">
-        <v>3827</v>
+        <v>735</v>
       </c>
     </row>
     <row r="12">
@@ -515,31 +509,9 @@
         <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>2285</v>
+        <v>103</v>
       </c>
       <c r="C12" t="n">
-        <v>1483</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="n">
-        <v>426</v>
-      </c>
-      <c r="C13" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" t="n">
-        <v>166</v>
-      </c>
-      <c r="C14" t="n">
         <v>0</v>
       </c>
     </row>
@@ -570,10 +542,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>0.295131721222845</v>
+        <v>0.280240952102234</v>
       </c>
       <c r="C2" t="n">
-        <v>0.227239832103054</v>
+        <v>0.36312799309914</v>
       </c>
     </row>
     <row r="3">
@@ -581,10 +553,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>0.139019954782267</v>
+        <v>0.14315676519364</v>
       </c>
       <c r="C3" t="n">
-        <v>0.10092426028162</v>
+        <v>0.0933400755525149</v>
       </c>
     </row>
     <row r="4">
@@ -592,10 +564,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.10220682197975</v>
+        <v>0.10839186420837</v>
       </c>
       <c r="C4" t="n">
-        <v>0.116473337055187</v>
+        <v>0.166007317290818</v>
       </c>
     </row>
     <row r="5">
@@ -603,10 +575,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>0.115821291654379</v>
+        <v>0.114671739342503</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0693505365672105</v>
+        <v>0.0596686397572801</v>
       </c>
     </row>
     <row r="6">
@@ -614,10 +586,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>0.0912341492185196</v>
+        <v>0.103782557799239</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0828939478526973</v>
+        <v>0.0519646628394658</v>
       </c>
     </row>
     <row r="7">
@@ -625,10 +597,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>0.0991226776762017</v>
+        <v>0.0947712418300654</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0451791658912805</v>
+        <v>0.00823938844106011</v>
       </c>
     </row>
     <row r="8">
@@ -636,10 +608,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0553057111963039</v>
+        <v>0.0620793093356746</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0720385418605132</v>
+        <v>0.0689193610755823</v>
       </c>
     </row>
     <row r="9">
@@ -647,10 +619,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0212203872997149</v>
+        <v>0.0225465808213833</v>
       </c>
       <c r="C9" t="n">
-        <v>0.108181874573538</v>
+        <v>0.121359945269044</v>
       </c>
     </row>
     <row r="10">
@@ -658,10 +630,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>0.0446156492676693</v>
+        <v>0.0428860598965955</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0678617951739967</v>
+        <v>0.0455099794758916</v>
       </c>
     </row>
     <row r="11">
@@ -669,10 +641,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>0.00097070677283004</v>
+        <v>0.0262169544434689</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0791307404420735</v>
+        <v>0.0218626371992028</v>
       </c>
     </row>
     <row r="12">
@@ -680,31 +652,9 @@
         <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>0.0280767718470461</v>
+        <v>0.00125597502682665</v>
       </c>
       <c r="C12" t="n">
-        <v>0.0306639373074458</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>14</v>
-      </c>
-      <c r="B13" t="n">
-        <v>0.00523444411677971</v>
-      </c>
-      <c r="C13" t="n">
-        <v>0.0000620308913839092</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" t="n">
-        <v>0.0020397129656935</v>
-      </c>
-      <c r="C14" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
MAST DE and UMAP overlays of genes of interest
</commit_message>
<xml_diff>
--- a/fullDataset/proportions/FLCvNML_cells_per_cluster.xlsx
+++ b/fullDataset/proportions/FLCvNML_cells_per_cluster.xlsx
@@ -399,10 +399,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>22982</v>
+        <v>24647</v>
       </c>
       <c r="C2" t="n">
-        <v>12208</v>
+        <v>12630</v>
       </c>
     </row>
     <row r="3">
@@ -410,10 +410,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>11740</v>
+        <v>11753</v>
       </c>
       <c r="C3" t="n">
-        <v>3138</v>
+        <v>3147</v>
       </c>
     </row>
     <row r="4">
@@ -421,10 +421,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>8889</v>
+        <v>7109</v>
       </c>
       <c r="C4" t="n">
-        <v>5581</v>
+        <v>4900</v>
       </c>
     </row>
     <row r="5">
@@ -432,10 +432,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>9404</v>
+        <v>9293</v>
       </c>
       <c r="C5" t="n">
-        <v>2006</v>
+        <v>1981</v>
       </c>
     </row>
     <row r="6">
@@ -443,10 +443,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>8511</v>
+        <v>8667</v>
       </c>
       <c r="C6" t="n">
-        <v>1747</v>
+        <v>1773</v>
       </c>
     </row>
     <row r="7">
@@ -454,10 +454,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>7772</v>
+        <v>7649</v>
       </c>
       <c r="C7" t="n">
-        <v>277</v>
+        <v>321</v>
       </c>
     </row>
     <row r="8">
@@ -465,10 +465,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>5091</v>
+        <v>5126</v>
       </c>
       <c r="C8" t="n">
-        <v>2317</v>
+        <v>2407</v>
       </c>
     </row>
     <row r="9">
@@ -476,10 +476,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>1849</v>
+        <v>1758</v>
       </c>
       <c r="C9" t="n">
-        <v>4080</v>
+        <v>4170</v>
       </c>
     </row>
     <row r="10">
@@ -487,10 +487,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>3517</v>
+        <v>3578</v>
       </c>
       <c r="C10" t="n">
-        <v>1530</v>
+        <v>1545</v>
       </c>
     </row>
     <row r="11">
@@ -498,10 +498,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>2150</v>
+        <v>2332</v>
       </c>
       <c r="C11" t="n">
-        <v>735</v>
+        <v>745</v>
       </c>
     </row>
     <row r="12">
@@ -509,7 +509,7 @@
         <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>
@@ -542,10 +542,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="n">
-        <v>0.280240952102234</v>
+        <v>0.300543849380548</v>
       </c>
       <c r="C2" t="n">
-        <v>0.36312799309914</v>
+        <v>0.375680418810792</v>
       </c>
     </row>
     <row r="3">
@@ -553,10 +553,10 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>0.14315676519364</v>
+        <v>0.14331528631353</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0933400755525149</v>
+        <v>0.0936077813141378</v>
       </c>
     </row>
     <row r="4">
@@ -564,10 +564,10 @@
         <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>0.10839186420837</v>
+        <v>0.0866866647156375</v>
       </c>
       <c r="C4" t="n">
-        <v>0.166007317290818</v>
+        <v>0.145750914661352</v>
       </c>
     </row>
     <row r="5">
@@ -575,10 +575,10 @@
         <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>0.114671739342503</v>
+        <v>0.113318212857282</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0596686397572801</v>
+        <v>0.058925012641661</v>
       </c>
     </row>
     <row r="6">
@@ -586,10 +586,10 @@
         <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>0.103782557799239</v>
+        <v>0.105684811237928</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0519646628394658</v>
+        <v>0.0527380350397097</v>
       </c>
     </row>
     <row r="7">
@@ -597,10 +597,10 @@
         <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>0.0947712418300654</v>
+        <v>0.093271388157253</v>
       </c>
       <c r="C7" t="n">
-        <v>0.00823938844106011</v>
+        <v>0.00954817216454981</v>
       </c>
     </row>
     <row r="8">
@@ -608,10 +608,10 @@
         <v>9</v>
       </c>
       <c r="B8" t="n">
-        <v>0.0620793093356746</v>
+        <v>0.0625060969661496</v>
       </c>
       <c r="C8" t="n">
-        <v>0.0689193610755823</v>
+        <v>0.0715964186918112</v>
       </c>
     </row>
     <row r="9">
@@ -619,10 +619,10 @@
         <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>0.0225465808213833</v>
+        <v>0.0214369329821481</v>
       </c>
       <c r="C9" t="n">
-        <v>0.121359945269044</v>
+        <v>0.124037002885273</v>
       </c>
     </row>
     <row r="10">
@@ -630,10 +630,10 @@
         <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>0.0428860598965955</v>
+        <v>0.043629889766852</v>
       </c>
       <c r="C10" t="n">
-        <v>0.0455099794758916</v>
+        <v>0.0459561557452631</v>
       </c>
     </row>
     <row r="11">
@@ -641,10 +641,10 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>0.0262169544434689</v>
+        <v>0.0284362501219393</v>
       </c>
       <c r="C11" t="n">
-        <v>0.0218626371992028</v>
+        <v>0.0221600880454505</v>
       </c>
     </row>
     <row r="12">
@@ -652,7 +652,7 @@
         <v>13</v>
       </c>
       <c r="B12" t="n">
-        <v>0.00125597502682665</v>
+        <v>0.00117061750073164</v>
       </c>
       <c r="C12" t="n">
         <v>0</v>

</xml_diff>